<commit_message>
wip(1d): pembanding paritas stok + berkas emas TS⇄Go (dua round2 TS ditiru)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/services/integrator/internal/document/testdata/kartu-stok-januari.golden.xlsx
+++ b/services/integrator/internal/document/testdata/kartu-stok-januari.golden.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t xml:space="preserve">PT Stok Uji</t>
   </si>
@@ -53,6 +53,9 @@
   </si>
   <si>
     <t xml:space="preserve">Gula Aren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kayu Manis</t>
   </si>
   <si>
     <t xml:space="preserve">Kopi Arabika</t>
@@ -330,10 +333,10 @@
         <v>12</v>
       </c>
       <c r="C10" s="7">
-        <v>7.625</v>
+        <v>0</v>
       </c>
       <c r="D10" s="7">
-        <v>4.875</v>
+        <v>0.5</v>
       </c>
       <c r="E10" s="7">
         <v>0</v>
@@ -342,30 +345,30 @@
         <v>0</v>
       </c>
       <c r="G10" s="7">
-        <v>12.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B11" t="s">
         <v>12</v>
       </c>
       <c r="C11" s="7">
-        <v>0</v>
+        <v>7.625</v>
       </c>
       <c r="D11" s="7">
-        <v>7</v>
+        <v>4.875</v>
       </c>
       <c r="E11" s="7">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F11" s="7">
         <v>0</v>
       </c>
       <c r="G11" s="7">
-        <v>0</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="12">
@@ -373,16 +376,16 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C12" s="7">
         <v>0</v>
       </c>
       <c r="D12" s="7">
-        <v>0.3</v>
+        <v>7</v>
       </c>
       <c r="E12" s="7">
-        <v>0.3</v>
+        <v>7</v>
       </c>
       <c r="F12" s="7">
         <v>0</v>
@@ -393,48 +396,48 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
         <v>18</v>
       </c>
-      <c r="B13" t="s">
-        <v>19</v>
-      </c>
       <c r="C13" s="7">
         <v>0</v>
       </c>
       <c r="D13" s="7">
-        <v>2</v>
+        <v>0.3</v>
       </c>
       <c r="E13" s="7">
-        <v>5.5</v>
+        <v>0.3</v>
       </c>
       <c r="F13" s="7">
         <v>0</v>
       </c>
       <c r="G13" s="7">
-        <v>-3.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" t="s">
         <v>20</v>
       </c>
-      <c r="B14" t="s">
-        <v>17</v>
-      </c>
       <c r="C14" s="7">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="D14" s="7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E14" s="7">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="F14" s="7">
         <v>0</v>
       </c>
       <c r="G14" s="7">
-        <v>1.25</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="15">
@@ -442,47 +445,70 @@
         <v>21</v>
       </c>
       <c r="B15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="7">
+        <v>1.25</v>
+      </c>
+      <c r="D15" s="7">
+        <v>0</v>
+      </c>
+      <c r="E15" s="7">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7">
+        <v>0</v>
+      </c>
+      <c r="G15" s="7">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="7">
-        <v>0</v>
-      </c>
-      <c r="D15" s="7">
+      <c r="B16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="7">
+        <v>0</v>
+      </c>
+      <c r="D16" s="7">
         <v>4</v>
       </c>
-      <c r="E15" s="7">
+      <c r="E16" s="7">
         <v>1</v>
       </c>
-      <c r="F15" s="7">
-        <v>0</v>
-      </c>
-      <c r="G15" s="7">
+      <c r="F16" s="7">
+        <v>0</v>
+      </c>
+      <c r="G16" s="7">
         <v>3</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="9">
+    <row r="17">
+      <c r="A17" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="9">
         <v>34.375</v>
       </c>
-      <c r="D16" s="9">
-        <v>168.175</v>
-      </c>
-      <c r="E16" s="9">
+      <c r="D17" s="9">
+        <v>168.675</v>
+      </c>
+      <c r="E17" s="9">
         <v>68.3</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F17" s="9">
         <v>5.25</v>
       </c>
-      <c r="G16" s="9">
-        <v>134.25</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s">
-        <v>24</v>
+      <c r="G17" s="9">
+        <v>134.75</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>